<commit_message>
feat: refactored visual 1 and added a 3rd visual
</commit_message>
<xml_diff>
--- a/Clemson Football Tickets  (Responses).xlsx
+++ b/Clemson Football Tickets  (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="166">
   <si>
     <t>Timestamp</t>
   </si>
@@ -501,6 +501,18 @@
   </si>
   <si>
     <t>Just give all students tickets who want them</t>
+  </si>
+  <si>
+    <t>Terrible and unfair</t>
+  </si>
+  <si>
+    <t>Not getting the games I want</t>
+  </si>
+  <si>
+    <t>They overprice</t>
+  </si>
+  <si>
+    <t>Less randomization and instead make it fair to earn the tickets, and also stop reselling of the tickets</t>
   </si>
 </sst>
 </file>
@@ -638,7 +650,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H40" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H41" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="8">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Do you participate in the Clemson Football Ticket Lottery? " id="2"/>
@@ -1891,6 +1903,32 @@
         <v>161</v>
       </c>
     </row>
+    <row r="41" ht="22.5" customHeight="1">
+      <c r="A41" s="5">
+        <v>46128.94800844908</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>